<commit_message>
uskorena logika rasscheta marshruta i gruppirovki
</commit_message>
<xml_diff>
--- a/TaxiLocations/employees.xlsx
+++ b/TaxiLocations/employees.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\simple\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93B677FF-3477-4064-9260-C26719E33812}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B462C9C3-7723-4652-B199-BF0224D27ED3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-4950" yWindow="-21720" windowWidth="38640" windowHeight="21840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="157">
   <si>
     <t>Id</t>
   </si>
@@ -148,9 +148,6 @@
     <t>Ахроробод 24</t>
   </si>
   <si>
-    <t>22:00:00</t>
-  </si>
-  <si>
     <t>Baxodirov Abdusattor</t>
   </si>
   <si>
@@ -187,9 +184,6 @@
     <t>Кўприклик, 107</t>
   </si>
   <si>
-    <t>nan</t>
-  </si>
-  <si>
     <t>Dunayev Danil Konstantinovich</t>
   </si>
   <si>
@@ -199,6 +193,12 @@
     <t>Dunayeva Olga</t>
   </si>
   <si>
+    <t>Djabbarova Sayyora Mamur qizi</t>
+  </si>
+  <si>
+    <t>4-й проезд Хосилот, 16</t>
+  </si>
+  <si>
     <t>Fatxullayev Sardor Muzaffar o'g'li</t>
   </si>
   <si>
@@ -361,9 +361,6 @@
     <t>Odrina Olesya</t>
   </si>
   <si>
-    <t>02:00:00</t>
-  </si>
-  <si>
     <t>Ostonaqulov Bilol</t>
   </si>
   <si>
@@ -484,23 +481,34 @@
     <t>Ибрат 68а</t>
   </si>
   <si>
-    <t>Djabbarova Sayyora Mamur qizi</t>
-  </si>
-  <si>
-    <t>4-й проезд Хосилот, 16</t>
+    <t>41.356346</t>
+  </si>
+  <si>
+    <t>69.220717</t>
+  </si>
+  <si>
+    <t>41.285319</t>
+  </si>
+  <si>
+    <t>69.248206</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -511,7 +519,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -519,12 +527,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -829,27 +855,30 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G73"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="29.44140625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1172,7 +1201,7 @@
         <v>69.241909000000007</v>
       </c>
       <c r="G15" t="s">
-        <v>42</v>
+        <v>17</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
@@ -1180,13 +1209,13 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D16" t="s">
         <v>43</v>
-      </c>
-      <c r="C16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D16" t="s">
-        <v>44</v>
       </c>
       <c r="E16">
         <v>41.325217000000002</v>
@@ -1203,19 +1232,19 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
+        <v>44</v>
+      </c>
+      <c r="C17" t="s">
+        <v>12</v>
+      </c>
+      <c r="D17" t="s">
         <v>45</v>
       </c>
-      <c r="C17" t="s">
-        <v>12</v>
-      </c>
-      <c r="D17" t="s">
-        <v>46</v>
-      </c>
       <c r="E17">
-        <v>41.328015000000001</v>
+        <v>41.318052000000002</v>
       </c>
       <c r="F17">
-        <v>69.239879999999999</v>
+        <v>69.224535000000003</v>
       </c>
       <c r="G17" t="s">
         <v>25</v>
@@ -1226,13 +1255,13 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
+        <v>46</v>
+      </c>
+      <c r="C18" t="s">
+        <v>8</v>
+      </c>
+      <c r="D18" t="s">
         <v>47</v>
-      </c>
-      <c r="C18" t="s">
-        <v>8</v>
-      </c>
-      <c r="D18" t="s">
-        <v>48</v>
       </c>
       <c r="E18">
         <v>41.245749000000004</v>
@@ -1249,13 +1278,13 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
+        <v>48</v>
+      </c>
+      <c r="C19" t="s">
+        <v>12</v>
+      </c>
+      <c r="D19" t="s">
         <v>49</v>
-      </c>
-      <c r="C19" t="s">
-        <v>12</v>
-      </c>
-      <c r="D19" t="s">
-        <v>50</v>
       </c>
       <c r="E19">
         <v>41.362316</v>
@@ -1272,13 +1301,13 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
+        <v>50</v>
+      </c>
+      <c r="C20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D20" t="s">
         <v>51</v>
-      </c>
-      <c r="C20" t="s">
-        <v>12</v>
-      </c>
-      <c r="D20" t="s">
-        <v>52</v>
       </c>
       <c r="E20">
         <v>41.302514000000002</v>
@@ -1295,22 +1324,19 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
+        <v>52</v>
+      </c>
+      <c r="C21" t="s">
+        <v>8</v>
+      </c>
+      <c r="D21" t="s">
         <v>53</v>
-      </c>
-      <c r="C21" t="s">
-        <v>8</v>
-      </c>
-      <c r="D21" t="s">
-        <v>54</v>
       </c>
       <c r="E21">
         <v>41.311143999999999</v>
       </c>
       <c r="F21">
         <v>69.279728000000006</v>
-      </c>
-      <c r="G21" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
@@ -1318,13 +1344,13 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C22" t="s">
         <v>12</v>
       </c>
       <c r="D22" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E22">
         <v>41.246712000000002</v>
@@ -1341,13 +1367,13 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C23" t="s">
         <v>8</v>
       </c>
       <c r="D23" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E23">
         <v>41.246712000000002</v>
@@ -1364,13 +1390,13 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>154</v>
+        <v>57</v>
       </c>
       <c r="C24" t="s">
         <v>8</v>
       </c>
       <c r="D24" t="s">
-        <v>155</v>
+        <v>58</v>
       </c>
       <c r="E24">
         <v>41.265909999999998</v>
@@ -1419,10 +1445,10 @@
         <v>62</v>
       </c>
       <c r="E26">
-        <v>41.281640000000003</v>
+        <v>41.297609999999999</v>
       </c>
       <c r="F26">
-        <v>69.339213999999998</v>
+        <v>69.360153999999994</v>
       </c>
       <c r="G26" t="s">
         <v>25</v>
@@ -1448,7 +1474,7 @@
         <v>69.339645000000004</v>
       </c>
       <c r="G27" t="s">
-        <v>55</v>
+        <v>14</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
@@ -1579,11 +1605,11 @@
       <c r="D33" t="s">
         <v>76</v>
       </c>
-      <c r="E33">
-        <v>41.355350999999999</v>
-      </c>
-      <c r="F33">
-        <v>69.218273999999994</v>
+      <c r="E33" t="s">
+        <v>153</v>
+      </c>
+      <c r="F33" t="s">
+        <v>154</v>
       </c>
       <c r="G33" t="s">
         <v>22</v>
@@ -1625,11 +1651,11 @@
       <c r="D35" t="s">
         <v>80</v>
       </c>
-      <c r="E35">
-        <v>41.311143999999999</v>
-      </c>
-      <c r="F35">
-        <v>69.279728000000006</v>
+      <c r="E35" t="s">
+        <v>155</v>
+      </c>
+      <c r="F35" t="s">
+        <v>156</v>
       </c>
       <c r="G35" t="s">
         <v>10</v>
@@ -1643,7 +1669,7 @@
         <v>81</v>
       </c>
       <c r="C36" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="D36" t="s">
         <v>82</v>
@@ -1655,7 +1681,7 @@
         <v>69.328734999999995</v>
       </c>
       <c r="G36" t="s">
-        <v>55</v>
+        <v>14</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.3">
@@ -1701,7 +1727,7 @@
         <v>69.229251000000005</v>
       </c>
       <c r="G38" t="s">
-        <v>55</v>
+        <v>14</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.3">
@@ -2023,7 +2049,7 @@
         <v>69.207243000000005</v>
       </c>
       <c r="G52" t="s">
-        <v>113</v>
+        <v>14</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.3">
@@ -2031,13 +2057,13 @@
         <v>52</v>
       </c>
       <c r="B53" t="s">
+        <v>113</v>
+      </c>
+      <c r="C53" t="s">
+        <v>12</v>
+      </c>
+      <c r="D53" t="s">
         <v>114</v>
-      </c>
-      <c r="C53" t="s">
-        <v>12</v>
-      </c>
-      <c r="D53" t="s">
-        <v>115</v>
       </c>
       <c r="E53">
         <v>41.269312999999997</v>
@@ -2054,13 +2080,13 @@
         <v>53</v>
       </c>
       <c r="B54" t="s">
+        <v>115</v>
+      </c>
+      <c r="C54" t="s">
+        <v>8</v>
+      </c>
+      <c r="D54" t="s">
         <v>116</v>
-      </c>
-      <c r="C54" t="s">
-        <v>12</v>
-      </c>
-      <c r="D54" t="s">
-        <v>117</v>
       </c>
       <c r="E54">
         <v>41.218271000000001</v>
@@ -2077,13 +2103,13 @@
         <v>54</v>
       </c>
       <c r="B55" t="s">
+        <v>117</v>
+      </c>
+      <c r="C55" t="s">
+        <v>8</v>
+      </c>
+      <c r="D55" t="s">
         <v>118</v>
-      </c>
-      <c r="C55" t="s">
-        <v>8</v>
-      </c>
-      <c r="D55" t="s">
-        <v>119</v>
       </c>
       <c r="E55">
         <v>41.214337</v>
@@ -2100,13 +2126,13 @@
         <v>55</v>
       </c>
       <c r="B56" t="s">
+        <v>119</v>
+      </c>
+      <c r="C56" t="s">
+        <v>12</v>
+      </c>
+      <c r="D56" t="s">
         <v>120</v>
-      </c>
-      <c r="C56" t="s">
-        <v>12</v>
-      </c>
-      <c r="D56" t="s">
-        <v>121</v>
       </c>
       <c r="E56">
         <v>41.334100999999997</v>
@@ -2123,13 +2149,13 @@
         <v>56</v>
       </c>
       <c r="B57" t="s">
+        <v>121</v>
+      </c>
+      <c r="C57" t="s">
+        <v>12</v>
+      </c>
+      <c r="D57" t="s">
         <v>122</v>
-      </c>
-      <c r="C57" t="s">
-        <v>12</v>
-      </c>
-      <c r="D57" t="s">
-        <v>123</v>
       </c>
       <c r="E57">
         <v>41.376899000000002</v>
@@ -2146,13 +2172,13 @@
         <v>57</v>
       </c>
       <c r="B58" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C58" t="s">
         <v>12</v>
       </c>
       <c r="D58" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E58">
         <v>41.376899000000002</v>
@@ -2169,13 +2195,13 @@
         <v>58</v>
       </c>
       <c r="B59" t="s">
+        <v>124</v>
+      </c>
+      <c r="C59" t="s">
+        <v>12</v>
+      </c>
+      <c r="D59" t="s">
         <v>125</v>
-      </c>
-      <c r="C59" t="s">
-        <v>12</v>
-      </c>
-      <c r="D59" t="s">
-        <v>126</v>
       </c>
       <c r="E59">
         <v>41.337764</v>
@@ -2192,13 +2218,13 @@
         <v>59</v>
       </c>
       <c r="B60" t="s">
+        <v>126</v>
+      </c>
+      <c r="C60" t="s">
+        <v>12</v>
+      </c>
+      <c r="D60" t="s">
         <v>127</v>
-      </c>
-      <c r="C60" t="s">
-        <v>12</v>
-      </c>
-      <c r="D60" t="s">
-        <v>128</v>
       </c>
       <c r="E60">
         <v>41.393203999999997</v>
@@ -2215,13 +2241,13 @@
         <v>60</v>
       </c>
       <c r="B61" t="s">
+        <v>128</v>
+      </c>
+      <c r="C61" t="s">
+        <v>8</v>
+      </c>
+      <c r="D61" t="s">
         <v>129</v>
-      </c>
-      <c r="C61" t="s">
-        <v>8</v>
-      </c>
-      <c r="D61" t="s">
-        <v>130</v>
       </c>
       <c r="E61">
         <v>41.240955999999997</v>
@@ -2238,13 +2264,13 @@
         <v>61</v>
       </c>
       <c r="B62" t="s">
+        <v>130</v>
+      </c>
+      <c r="C62" t="s">
+        <v>8</v>
+      </c>
+      <c r="D62" t="s">
         <v>131</v>
-      </c>
-      <c r="C62" t="s">
-        <v>8</v>
-      </c>
-      <c r="D62" t="s">
-        <v>132</v>
       </c>
       <c r="E62">
         <v>41.211508000000002</v>
@@ -2261,13 +2287,13 @@
         <v>62</v>
       </c>
       <c r="B63" t="s">
+        <v>132</v>
+      </c>
+      <c r="C63" t="s">
+        <v>12</v>
+      </c>
+      <c r="D63" t="s">
         <v>133</v>
-      </c>
-      <c r="C63" t="s">
-        <v>12</v>
-      </c>
-      <c r="D63" t="s">
-        <v>134</v>
       </c>
       <c r="E63">
         <v>41.311475999999999</v>
@@ -2284,13 +2310,13 @@
         <v>63</v>
       </c>
       <c r="B64" t="s">
+        <v>134</v>
+      </c>
+      <c r="C64" t="s">
+        <v>12</v>
+      </c>
+      <c r="D64" t="s">
         <v>135</v>
-      </c>
-      <c r="C64" t="s">
-        <v>12</v>
-      </c>
-      <c r="D64" t="s">
-        <v>136</v>
       </c>
       <c r="E64">
         <v>41.2804</v>
@@ -2307,13 +2333,13 @@
         <v>64</v>
       </c>
       <c r="B65" t="s">
+        <v>136</v>
+      </c>
+      <c r="C65" t="s">
+        <v>12</v>
+      </c>
+      <c r="D65" t="s">
         <v>137</v>
-      </c>
-      <c r="C65" t="s">
-        <v>12</v>
-      </c>
-      <c r="D65" t="s">
-        <v>138</v>
       </c>
       <c r="E65">
         <v>41.268146999999999</v>
@@ -2330,13 +2356,13 @@
         <v>65</v>
       </c>
       <c r="B66" t="s">
+        <v>138</v>
+      </c>
+      <c r="C66" t="s">
+        <v>12</v>
+      </c>
+      <c r="D66" t="s">
         <v>139</v>
-      </c>
-      <c r="C66" t="s">
-        <v>12</v>
-      </c>
-      <c r="D66" t="s">
-        <v>140</v>
       </c>
       <c r="E66">
         <v>41.361964</v>
@@ -2353,22 +2379,19 @@
         <v>66</v>
       </c>
       <c r="B67" t="s">
+        <v>140</v>
+      </c>
+      <c r="C67" t="s">
+        <v>8</v>
+      </c>
+      <c r="D67" t="s">
         <v>141</v>
-      </c>
-      <c r="C67" t="s">
-        <v>8</v>
-      </c>
-      <c r="D67" t="s">
-        <v>142</v>
       </c>
       <c r="E67">
         <v>41.361320999999997</v>
       </c>
       <c r="F67">
         <v>69.286725000000004</v>
-      </c>
-      <c r="G67" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.3">
@@ -2376,13 +2399,13 @@
         <v>67</v>
       </c>
       <c r="B68" t="s">
+        <v>142</v>
+      </c>
+      <c r="C68" t="s">
+        <v>12</v>
+      </c>
+      <c r="D68" t="s">
         <v>143</v>
-      </c>
-      <c r="C68" t="s">
-        <v>12</v>
-      </c>
-      <c r="D68" t="s">
-        <v>144</v>
       </c>
       <c r="E68">
         <v>41.252780000000001</v>
@@ -2399,13 +2422,13 @@
         <v>68</v>
       </c>
       <c r="B69" t="s">
+        <v>144</v>
+      </c>
+      <c r="C69" t="s">
+        <v>12</v>
+      </c>
+      <c r="D69" t="s">
         <v>145</v>
-      </c>
-      <c r="C69" t="s">
-        <v>12</v>
-      </c>
-      <c r="D69" t="s">
-        <v>146</v>
       </c>
       <c r="E69">
         <v>41.335664999999999</v>
@@ -2414,7 +2437,7 @@
         <v>69.371561999999997</v>
       </c>
       <c r="G69" t="s">
-        <v>55</v>
+        <v>14</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.3">
@@ -2422,13 +2445,13 @@
         <v>69</v>
       </c>
       <c r="B70" t="s">
+        <v>146</v>
+      </c>
+      <c r="C70" t="s">
+        <v>8</v>
+      </c>
+      <c r="D70" t="s">
         <v>147</v>
-      </c>
-      <c r="C70" t="s">
-        <v>8</v>
-      </c>
-      <c r="D70" t="s">
-        <v>148</v>
       </c>
       <c r="E70">
         <v>41.355676000000003</v>
@@ -2445,13 +2468,13 @@
         <v>70</v>
       </c>
       <c r="B71" t="s">
+        <v>148</v>
+      </c>
+      <c r="C71" t="s">
+        <v>12</v>
+      </c>
+      <c r="D71" t="s">
         <v>149</v>
-      </c>
-      <c r="C71" t="s">
-        <v>12</v>
-      </c>
-      <c r="D71" t="s">
-        <v>150</v>
       </c>
       <c r="E71">
         <v>41.409613</v>
@@ -2468,13 +2491,13 @@
         <v>71</v>
       </c>
       <c r="B72" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C72" t="s">
         <v>8</v>
       </c>
       <c r="D72" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E72">
         <v>41.409613</v>
@@ -2491,13 +2514,13 @@
         <v>72</v>
       </c>
       <c r="B73" t="s">
+        <v>151</v>
+      </c>
+      <c r="C73" t="s">
+        <v>12</v>
+      </c>
+      <c r="D73" t="s">
         <v>152</v>
-      </c>
-      <c r="C73" t="s">
-        <v>12</v>
-      </c>
-      <c r="D73" t="s">
-        <v>153</v>
       </c>
       <c r="E73">
         <v>41.308081999999999</v>
@@ -2510,9 +2533,6 @@
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:A73">
-    <sortCondition ref="A2:A73"/>
-  </sortState>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>